<commit_message>
vault backup: 2026-10-13 20:47:48
</commit_message>
<xml_diff>
--- a/ПРЕДМЕТЫ/Методологии и проектирование ИС/ДЗ/Л2/ЛР_2_Поповкин_таблицы.xlsx
+++ b/ПРЕДМЕТЫ/Методологии и проектирование ИС/ДЗ/Л2/ЛР_2_Поповкин_таблицы.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\GitHub\obsidian-dvfu_p2\ПРЕДМЕТЫ\Методологии и проектирование ИС\ДЗ\Л2\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8ABFA621-54FC-4820-91A3-7532CD52B6ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -18,14 +24,128 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="28">
+  <si>
+    <t>Перекрестки</t>
+  </si>
+  <si>
+    <t>Наименование (Название блока)</t>
+  </si>
+  <si>
+    <t>Описание (Назначение операции)</t>
+  </si>
+  <si>
+    <t>Аккуратный демонтаж корпуса и внутренних узлов устройства для обеспечения физического доступа к поврежденным компонентам.</t>
+  </si>
+  <si>
+    <t>Физическое устранение поломки: пайка, замена вышедших из строя микросхем, конденсаторов, шлейфов или механических частей.</t>
+  </si>
+  <si>
+    <t>Устранение программных сбоев: перепрошивка BIOS/UEFI, обновление микрокода, сброс ошибок контроллеров.</t>
+  </si>
+  <si>
+    <t>Обратная сборка устройства, замена термоинтерфейса (термопасты/термопрокладок), очистка от пыли и подготовка к включению.</t>
+  </si>
+  <si>
+    <t>Фиксация факта выполненных работ и использованных запчастей в учетной системе (CRM) и физическая передача устройства на выходное тестирование.</t>
+  </si>
+  <si>
+    <t>Процессы (работы) диаграммы</t>
+  </si>
+  <si>
+    <t>J2</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> J3</t>
+  </si>
+  <si>
+    <t>№</t>
+  </si>
+  <si>
+    <t>Асинхронное ИЛИ</t>
+  </si>
+  <si>
+    <t>Разборка и подготовка</t>
+  </si>
+  <si>
+    <t>Аппаратное восстановление</t>
+  </si>
+  <si>
+    <t>Программное восстановление</t>
+  </si>
+  <si>
+    <t>Сборка и профилактика</t>
+  </si>
+  <si>
+    <t>Оформление и передача на ОТК</t>
+  </si>
+  <si>
+    <t>Наименование процессов слияния</t>
+  </si>
+  <si>
+    <t>Наименование процессов разветвления</t>
+  </si>
+  <si>
+    <t>Тип перекрёстка</t>
+  </si>
+  <si>
+    <t>Описание (назначение)</t>
+  </si>
+  <si>
+    <t>—</t>
+  </si>
+  <si>
+    <t>Синхронное И</t>
+  </si>
+  <si>
+    <t>Ветвление процесса. Разделение потока работ в зависимости от характера выявленных неисправностей. Допускается выполнение как одного из видов ремонта, так и обоих параллельно (или последовательно) в случае комбинированной поломки устройства.</t>
+  </si>
+  <si>
+    <t>Слияние потоков. Жёсткое условие: переход к этапу сборки и финальной профилактики возможен только после полного завершения всех запланированных работ по восстановлению (и аппаратных, и программных).</t>
+  </si>
+  <si>
+    <t>«Аппаратное восстановление», «Программное восстановление» — «Сборка и профилактика»</t>
+  </si>
+  <si>
+    <t>«Разборка и подготовка»  — «Аппаратное восстановление», «Программное восстановление»</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -37,7 +157,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,15 +165,44 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  <cellStyles count="2">
+    <cellStyle name="Обычный" xfId="0" builtinId="0"/>
+    <cellStyle name="Обычный 2" xfId="1" xr:uid="{E9040072-210D-4185-8E5E-A91B779BDA27}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -330,10 +479,136 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:E13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="24.42578125" customWidth="1"/>
+    <col min="2" max="2" width="74.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="38.42578125" customWidth="1"/>
+    <col min="4" max="4" width="15.7109375" customWidth="1"/>
+    <col min="5" max="5" width="43.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="4"/>
+    </row>
+    <row r="2" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A10" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B10" s="4"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4"/>
+    </row>
+    <row r="11" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="113.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="113.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A10:E10"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>